<commit_message>
re-export results to excel
</commit_message>
<xml_diff>
--- a/experiments/nrp_sat_adder_exp_results.xlsx
+++ b/experiments/nrp_sat_adder_exp_results.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,30 +447,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>encoding_time_sec</t>
+          <t>total_time_sec</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>solving_time_sec</t>
+          <t>peak_memory_mb</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>total_time_sec</t>
+          <t>total_clauses</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>peak_memory_mb</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_clauses</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>total_variables</t>
         </is>
@@ -495,21 +485,15 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.185631</v>
+        <v>0.189716</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00408479</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>0.189716</v>
+        <v>18143</v>
       </c>
       <c r="I2" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="J2" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K2" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -532,21 +516,15 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.188883</v>
+        <v>0.193092</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00420899</v>
+        <v>9.4</v>
       </c>
       <c r="H3" t="n">
-        <v>0.193092</v>
+        <v>18143</v>
       </c>
       <c r="I3" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="J3" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K3" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -569,21 +547,15 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.189249</v>
+        <v>0.193438</v>
       </c>
       <c r="G4" t="n">
-        <v>0.00418891</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>0.193438</v>
+        <v>18143</v>
       </c>
       <c r="I4" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J4" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K4" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -606,21 +578,15 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.190338</v>
+        <v>0.194484</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0041455</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>0.194484</v>
+        <v>18143</v>
       </c>
       <c r="I5" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J5" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K5" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -643,21 +609,15 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.189466</v>
+        <v>0.19343</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00396406</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.19343</v>
+        <v>18143</v>
       </c>
       <c r="I6" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J6" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K6" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -680,21 +640,15 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.190059</v>
+        <v>0.19429</v>
       </c>
       <c r="G7" t="n">
-        <v>0.00423078</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>0.19429</v>
+        <v>18143</v>
       </c>
       <c r="I7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J7" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K7" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -717,21 +671,15 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.187692</v>
+        <v>0.191775</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00408295</v>
+        <v>9.4</v>
       </c>
       <c r="H8" t="n">
-        <v>0.191775</v>
+        <v>18143</v>
       </c>
       <c r="I8" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="J8" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K8" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -754,21 +702,15 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.185392</v>
+        <v>0.189465</v>
       </c>
       <c r="G9" t="n">
-        <v>0.00407283</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>0.189465</v>
+        <v>18143</v>
       </c>
       <c r="I9" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="J9" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K9" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -791,21 +733,15 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.188961</v>
+        <v>0.1932</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00423961</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1932</v>
+        <v>18143</v>
       </c>
       <c r="I10" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="J10" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K10" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -828,21 +764,15 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.187664</v>
+        <v>0.191707</v>
       </c>
       <c r="G11" t="n">
-        <v>0.00404308</v>
+        <v>9.4</v>
       </c>
       <c r="H11" t="n">
-        <v>0.191707</v>
+        <v>18143</v>
       </c>
       <c r="I11" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="J11" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K11" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -867,21 +797,15 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1883335</v>
+        <v>0.1924597</v>
       </c>
       <c r="G12" t="n">
-        <v>0.00412615</v>
+        <v>9.570000000000002</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1924597</v>
+        <v>18143</v>
       </c>
       <c r="I12" t="n">
-        <v>9.570000000000002</v>
-      </c>
-      <c r="J12" t="n">
-        <v>18143</v>
-      </c>
-      <c r="K12" t="n">
         <v>8525</v>
       </c>
     </row>
@@ -896,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -927,30 +851,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>encoding_time_sec</t>
+          <t>total_time_sec</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>solving_time_sec</t>
+          <t>peak_memory_mb</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>total_time_sec</t>
+          <t>total_clauses</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>peak_memory_mb</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_clauses</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>total_variables</t>
         </is>
@@ -975,21 +889,15 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.298343</v>
+        <v>0.305666</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0073228</v>
+        <v>15.2</v>
       </c>
       <c r="H2" t="n">
-        <v>0.305666</v>
+        <v>33803</v>
       </c>
       <c r="I2" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="J2" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K2" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1012,21 +920,15 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.293668</v>
+        <v>0.300536</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00686736</v>
+        <v>14.9</v>
       </c>
       <c r="H3" t="n">
-        <v>0.300536</v>
+        <v>33803</v>
       </c>
       <c r="I3" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J3" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K3" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1049,21 +951,15 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.293914</v>
+        <v>0.301325</v>
       </c>
       <c r="G4" t="n">
-        <v>0.00741162</v>
+        <v>14.9</v>
       </c>
       <c r="H4" t="n">
-        <v>0.301325</v>
+        <v>33803</v>
       </c>
       <c r="I4" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J4" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K4" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1086,21 +982,15 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.29466</v>
+        <v>0.301665</v>
       </c>
       <c r="G5" t="n">
-        <v>0.00700498</v>
+        <v>14.9</v>
       </c>
       <c r="H5" t="n">
-        <v>0.301665</v>
+        <v>33803</v>
       </c>
       <c r="I5" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J5" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K5" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1123,21 +1013,15 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.294116</v>
+        <v>0.301101</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00698416</v>
+        <v>14.9</v>
       </c>
       <c r="H6" t="n">
-        <v>0.301101</v>
+        <v>33803</v>
       </c>
       <c r="I6" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J6" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K6" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1160,21 +1044,15 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.294341</v>
+        <v>0.301417</v>
       </c>
       <c r="G7" t="n">
-        <v>0.00707638</v>
+        <v>14.8</v>
       </c>
       <c r="H7" t="n">
-        <v>0.301417</v>
+        <v>33803</v>
       </c>
       <c r="I7" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="J7" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K7" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1197,21 +1075,15 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.292772</v>
+        <v>0.299767</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0069949</v>
+        <v>15.2</v>
       </c>
       <c r="H8" t="n">
-        <v>0.299767</v>
+        <v>33803</v>
       </c>
       <c r="I8" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="J8" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K8" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1234,21 +1106,15 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.29342</v>
+        <v>0.300448</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0070282</v>
+        <v>14.9</v>
       </c>
       <c r="H9" t="n">
-        <v>0.300448</v>
+        <v>33803</v>
       </c>
       <c r="I9" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J9" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K9" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1271,21 +1137,15 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.296001</v>
+        <v>0.302976</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00697503</v>
+        <v>15.2</v>
       </c>
       <c r="H10" t="n">
-        <v>0.302976</v>
+        <v>33803</v>
       </c>
       <c r="I10" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="J10" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K10" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1308,21 +1168,15 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.295417</v>
+        <v>0.302566</v>
       </c>
       <c r="G11" t="n">
-        <v>0.00714928</v>
+        <v>14.9</v>
       </c>
       <c r="H11" t="n">
-        <v>0.302566</v>
+        <v>33803</v>
       </c>
       <c r="I11" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="J11" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K11" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1347,21 +1201,15 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2946652</v>
+        <v>0.3017467</v>
       </c>
       <c r="G12" t="n">
-        <v>0.007081470999999999</v>
+        <v>14.98</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3017467</v>
+        <v>33803</v>
       </c>
       <c r="I12" t="n">
-        <v>14.98</v>
-      </c>
-      <c r="J12" t="n">
-        <v>33803</v>
-      </c>
-      <c r="K12" t="n">
         <v>15745</v>
       </c>
     </row>
@@ -1376,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1407,30 +1255,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>encoding_time_sec</t>
+          <t>total_time_sec</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>solving_time_sec</t>
+          <t>peak_memory_mb</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>total_time_sec</t>
+          <t>total_clauses</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>peak_memory_mb</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_clauses</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>total_variables</t>
         </is>
@@ -1455,21 +1293,15 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.405171</v>
+        <v>0.415687</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0105159</v>
+        <v>19.4</v>
       </c>
       <c r="H2" t="n">
-        <v>0.415687</v>
+        <v>49463</v>
       </c>
       <c r="I2" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="J2" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K2" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1492,21 +1324,15 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.416588</v>
+        <v>0.427761</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0111727</v>
+        <v>19.3</v>
       </c>
       <c r="H3" t="n">
-        <v>0.427761</v>
+        <v>49463</v>
       </c>
       <c r="I3" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J3" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K3" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1529,21 +1355,15 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.402766</v>
+        <v>0.414635</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0118691</v>
+        <v>19.3</v>
       </c>
       <c r="H4" t="n">
-        <v>0.414635</v>
+        <v>49463</v>
       </c>
       <c r="I4" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J4" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K4" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1566,21 +1386,15 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.403212</v>
+        <v>0.413647</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0104348</v>
+        <v>19.4</v>
       </c>
       <c r="H5" t="n">
-        <v>0.413647</v>
+        <v>49463</v>
       </c>
       <c r="I5" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="J5" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K5" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1603,21 +1417,15 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.40112</v>
+        <v>0.411767</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0106473</v>
+        <v>19.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.411767</v>
+        <v>49463</v>
       </c>
       <c r="I6" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J6" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K6" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1640,21 +1448,15 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.41883</v>
+        <v>0.429422</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0105926</v>
+        <v>19.3</v>
       </c>
       <c r="H7" t="n">
-        <v>0.429422</v>
+        <v>49463</v>
       </c>
       <c r="I7" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J7" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K7" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1677,21 +1479,15 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.411193</v>
+        <v>0.422219</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0110254</v>
+        <v>19.3</v>
       </c>
       <c r="H8" t="n">
-        <v>0.422219</v>
+        <v>49463</v>
       </c>
       <c r="I8" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J8" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K8" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1714,21 +1510,15 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.407128</v>
+        <v>0.417983</v>
       </c>
       <c r="G9" t="n">
-        <v>0.010855</v>
+        <v>19.3</v>
       </c>
       <c r="H9" t="n">
-        <v>0.417983</v>
+        <v>49463</v>
       </c>
       <c r="I9" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J9" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K9" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1751,21 +1541,15 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.40564</v>
+        <v>0.416378</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0107382</v>
+        <v>19.3</v>
       </c>
       <c r="H10" t="n">
-        <v>0.416378</v>
+        <v>49463</v>
       </c>
       <c r="I10" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J10" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K10" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1788,21 +1572,15 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.408483</v>
+        <v>0.418874</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0103909</v>
+        <v>19.3</v>
       </c>
       <c r="H11" t="n">
-        <v>0.418874</v>
+        <v>49463</v>
       </c>
       <c r="I11" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J11" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K11" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1827,21 +1605,15 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4080131000000001</v>
+        <v>0.4188373</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01082419</v>
+        <v>19.32</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4188373</v>
+        <v>49463</v>
       </c>
       <c r="I12" t="n">
-        <v>19.32</v>
-      </c>
-      <c r="J12" t="n">
-        <v>49463</v>
-      </c>
-      <c r="K12" t="n">
         <v>22965</v>
       </c>
     </row>
@@ -1856,7 +1628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1887,30 +1659,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>encoding_time_sec</t>
+          <t>total_time_sec</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>solving_time_sec</t>
+          <t>peak_memory_mb</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>total_time_sec</t>
+          <t>total_clauses</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>peak_memory_mb</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_clauses</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>total_variables</t>
         </is>
@@ -1935,21 +1697,15 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.514954</v>
+        <v>0.5287809999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0138271</v>
+        <v>26.1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5287809999999999</v>
+        <v>65123</v>
       </c>
       <c r="I2" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K2" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -1972,21 +1728,15 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.513867</v>
+        <v>0.528764</v>
       </c>
       <c r="G3" t="n">
-        <v>0.014897</v>
+        <v>26.6</v>
       </c>
       <c r="H3" t="n">
-        <v>0.528764</v>
+        <v>65123</v>
       </c>
       <c r="I3" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="J3" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K3" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2009,21 +1759,15 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.533424</v>
+        <v>0.547589</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0141651</v>
+        <v>26.6</v>
       </c>
       <c r="H4" t="n">
-        <v>0.547589</v>
+        <v>65123</v>
       </c>
       <c r="I4" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="J4" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K4" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2046,21 +1790,15 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.52912</v>
+        <v>0.543646</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0145266</v>
+        <v>26.7</v>
       </c>
       <c r="H5" t="n">
-        <v>0.543646</v>
+        <v>65123</v>
       </c>
       <c r="I5" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="J5" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K5" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2083,21 +1821,15 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.510758</v>
+        <v>0.524801</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0140437</v>
+        <v>26.2</v>
       </c>
       <c r="H6" t="n">
-        <v>0.524801</v>
+        <v>65123</v>
       </c>
       <c r="I6" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J6" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K6" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2120,21 +1852,15 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5200129999999999</v>
+        <v>0.534262</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0142488</v>
+        <v>26.1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.534262</v>
+        <v>65123</v>
       </c>
       <c r="I7" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K7" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2157,21 +1883,15 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.529208</v>
+        <v>0.54337</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0141616</v>
+        <v>26.1</v>
       </c>
       <c r="H8" t="n">
-        <v>0.54337</v>
+        <v>65123</v>
       </c>
       <c r="I8" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K8" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2194,21 +1914,15 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.516948</v>
+        <v>0.531254</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0143065</v>
+        <v>26.6</v>
       </c>
       <c r="H9" t="n">
-        <v>0.531254</v>
+        <v>65123</v>
       </c>
       <c r="I9" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="J9" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K9" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2231,21 +1945,15 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.51892</v>
+        <v>0.533131</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0142111</v>
+        <v>26.5</v>
       </c>
       <c r="H10" t="n">
-        <v>0.533131</v>
+        <v>65123</v>
       </c>
       <c r="I10" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="J10" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K10" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2268,21 +1976,15 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.519026</v>
+        <v>0.5329930000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>0.013967</v>
+        <v>26.6</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5329930000000001</v>
+        <v>65123</v>
       </c>
       <c r="I11" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="J11" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K11" t="n">
         <v>30185</v>
       </c>
     </row>
@@ -2307,21 +2009,15 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5206237999999999</v>
+        <v>0.5348591</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01423545</v>
+        <v>26.41</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5348591</v>
+        <v>65123</v>
       </c>
       <c r="I12" t="n">
-        <v>26.41</v>
-      </c>
-      <c r="J12" t="n">
-        <v>65123</v>
-      </c>
-      <c r="K12" t="n">
         <v>30185</v>
       </c>
     </row>

</xml_diff>